<commit_message>
Cerrar el S2 en el Sprint Backlog
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/RecyTrack_Sprint_Backlog.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/RecyTrack_Sprint_Backlog.xlsx
@@ -5312,8 +5312,10 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
-        <v>47</v>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Las historias de cada sprint vienen del Product Backlog. Las que quedan para después del piloto no se asignan a ningún sprint. En el S2 se terminaron también historias planificadas para S3, S4 y S5; en sus hojas aparecen como Hecho con la fecha real.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -6616,8 +6618,10 @@
       <c r="A6" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>183</v>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cerrado</t>
+        </is>
       </c>
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
@@ -6733,13 +6737,19 @@
       <c r="D12" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="E12" s="17"/>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vicente Torres y Álvaro Jaña</t>
+        </is>
+      </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G12" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>46301</v>
+      </c>
       <c r="H12" s="5" t="s">
         <v>191</v>
       </c>
@@ -6754,7 +6764,6 @@
         <v>31</v>
       </c>
       <c r="M12" s="4" t="n">
-        <f aca="false">$B$7</f>
         <v>31</v>
       </c>
       <c r="N12" s="4" t="n">
@@ -6775,11 +6784,19 @@
       <c r="D13" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E13" s="17"/>
-      <c r="F13" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="G13" s="19"/>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H13" s="5" t="s">
         <v>194</v>
       </c>
@@ -6793,7 +6810,9 @@
         <f aca="false">$B$7*(9-J13)/8</f>
         <v>27.125</v>
       </c>
-      <c r="M13" s="6"/>
+      <c r="M13" s="6" t="n">
+        <v>23</v>
+      </c>
       <c r="N13" s="4" t="n">
         <f aca="false">$B$7-SUMIFS($D$12:$D$18,$F$12:$F$18,"Hecho",$G$12:$G$18,"&lt;="&amp;K13)</f>
         <v>31</v>
@@ -6812,13 +6831,19 @@
       <c r="D14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="17"/>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G14" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H14" s="5" t="s">
         <v>197</v>
       </c>
@@ -6832,7 +6857,9 @@
         <f aca="false">$B$7*(9-J14)/8</f>
         <v>23.25</v>
       </c>
-      <c r="M14" s="6"/>
+      <c r="M14" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="N14" s="4" t="n">
         <f aca="false">$B$7-SUMIFS($D$12:$D$18,$F$12:$F$18,"Hecho",$G$12:$G$18,"&lt;="&amp;K14)</f>
         <v>31</v>
@@ -6851,11 +6878,19 @@
       <c r="D15" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E15" s="17"/>
-      <c r="F15" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="G15" s="19"/>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G15" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H15" s="5" t="s">
         <v>200</v>
       </c>
@@ -6869,7 +6904,9 @@
         <f aca="false">$B$7*(9-J15)/8</f>
         <v>19.375</v>
       </c>
-      <c r="M15" s="6"/>
+      <c r="M15" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="N15" s="4" t="n">
         <f aca="false">$B$7-SUMIFS($D$12:$D$18,$F$12:$F$18,"Hecho",$G$12:$G$18,"&lt;="&amp;K15)</f>
         <v>31</v>
@@ -6888,13 +6925,19 @@
       <c r="D16" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E16" s="17"/>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G16" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G16" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H16" s="5" t="s">
         <v>203</v>
       </c>
@@ -6908,7 +6951,9 @@
         <f aca="false">$B$7*(9-J16)/8</f>
         <v>15.5</v>
       </c>
-      <c r="M16" s="6"/>
+      <c r="M16" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="N16" s="4" t="n">
         <f aca="false">$B$7-SUMIFS($D$12:$D$18,$F$12:$F$18,"Hecho",$G$12:$G$18,"&lt;="&amp;K16)</f>
         <v>31</v>
@@ -6927,13 +6972,19 @@
       <c r="D17" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E17" s="17"/>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G17" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G17" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H17" s="5" t="s">
         <v>206</v>
       </c>
@@ -6947,7 +6998,9 @@
         <f aca="false">$B$7*(9-J17)/8</f>
         <v>11.625</v>
       </c>
-      <c r="M17" s="6"/>
+      <c r="M17" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="N17" s="4" t="n">
         <f aca="false">$B$7-SUMIFS($D$12:$D$18,$F$12:$F$18,"Hecho",$G$12:$G$18,"&lt;="&amp;K17)</f>
         <v>31</v>
@@ -6966,11 +7019,19 @@
       <c r="D18" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E18" s="17"/>
-      <c r="F18" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="G18" s="19"/>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G18" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H18" s="5" t="s">
         <v>209</v>
       </c>
@@ -6984,7 +7045,9 @@
         <f aca="false">$B$7*(9-J18)/8</f>
         <v>7.75</v>
       </c>
-      <c r="M18" s="6"/>
+      <c r="M18" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="N18" s="4" t="n">
         <f aca="false">$B$7-SUMIFS($D$12:$D$18,$F$12:$F$18,"Hecho",$G$12:$G$18,"&lt;="&amp;K18)</f>
         <v>31</v>
@@ -7001,7 +7064,9 @@
         <f aca="false">$B$7*(9-J19)/8</f>
         <v>3.875</v>
       </c>
-      <c r="M19" s="6"/>
+      <c r="M19" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="N19" s="4" t="n">
         <f aca="false">$B$7-SUMIFS($D$12:$D$18,$F$12:$F$18,"Hecho",$G$12:$G$18,"&lt;="&amp;K19)</f>
         <v>31</v>
@@ -7021,7 +7086,9 @@
         <f aca="false">$B$7*(9-J20)/8</f>
         <v>0</v>
       </c>
-      <c r="M20" s="6"/>
+      <c r="M20" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="N20" s="4" t="n">
         <f aca="false">$B$7-SUMIFS($D$12:$D$18,$F$12:$F$18,"Hecho",$G$12:$G$18,"&lt;="&amp;K20)</f>
         <v>31</v>
@@ -7207,14 +7274,24 @@
         <v>192</v>
       </c>
       <c r="D27" s="6"/>
-      <c r="E27" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G27" s="19"/>
-      <c r="H27" s="17"/>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G27" s="19" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H27" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PR #43</t>
+        </is>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
@@ -7227,14 +7304,24 @@
         <v>192</v>
       </c>
       <c r="D28" s="6"/>
-      <c r="E28" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="F28" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G28" s="19"/>
-      <c r="H28" s="17"/>
+      <c r="E28" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G28" s="19" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H28" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PR #43</t>
+        </is>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
@@ -7247,14 +7334,24 @@
         <v>192</v>
       </c>
       <c r="D29" s="6"/>
-      <c r="E29" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G29" s="19"/>
-      <c r="H29" s="17"/>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G29" s="19" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H29" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PR #43</t>
+        </is>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
@@ -7267,14 +7364,24 @@
         <v>195</v>
       </c>
       <c r="D30" s="6"/>
-      <c r="E30" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="F30" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G30" s="19"/>
-      <c r="H30" s="17"/>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G30" s="19" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H30" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PR #44</t>
+        </is>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
@@ -7287,14 +7394,24 @@
         <v>195</v>
       </c>
       <c r="D31" s="6"/>
-      <c r="E31" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G31" s="19"/>
-      <c r="H31" s="17"/>
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G31" s="19" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H31" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PR #44</t>
+        </is>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
@@ -7310,11 +7427,17 @@
       <c r="E32" s="17" t="s">
         <v>213</v>
       </c>
-      <c r="F32" s="6" t="s">
-        <v>214</v>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Por hacer</t>
+        </is>
       </c>
       <c r="G32" s="19"/>
-      <c r="H32" s="17"/>
+      <c r="H32" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Las reglas no verifican que el código del área no se repita; pasa al S3</t>
+        </is>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
@@ -7327,14 +7450,24 @@
         <v>198</v>
       </c>
       <c r="D33" s="6"/>
-      <c r="E33" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G33" s="19"/>
-      <c r="H33" s="17"/>
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G33" s="19" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H33" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PR #44</t>
+        </is>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
@@ -7347,14 +7480,24 @@
         <v>198</v>
       </c>
       <c r="D34" s="6"/>
-      <c r="E34" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="F34" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G34" s="19"/>
-      <c r="H34" s="17"/>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G34" s="19" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H34" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PR #44</t>
+        </is>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
@@ -7367,14 +7510,24 @@
         <v>198</v>
       </c>
       <c r="D35" s="6"/>
-      <c r="E35" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="F35" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G35" s="19"/>
-      <c r="H35" s="17"/>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G35" s="19" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H35" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PR #44</t>
+        </is>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
@@ -7387,14 +7540,24 @@
         <v>201</v>
       </c>
       <c r="D36" s="6"/>
-      <c r="E36" s="17" t="s">
-        <v>213</v>
-      </c>
-      <c r="F36" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G36" s="19"/>
-      <c r="H36" s="17"/>
+      <c r="E36" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G36" s="19" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H36" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PR #44</t>
+        </is>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
@@ -7407,14 +7570,24 @@
         <v>201</v>
       </c>
       <c r="D37" s="6"/>
-      <c r="E37" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="F37" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G37" s="19"/>
-      <c r="H37" s="17"/>
+      <c r="E37" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G37" s="19" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H37" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PR #44</t>
+        </is>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
@@ -7427,18 +7600,22 @@
         <v>201</v>
       </c>
       <c r="D38" s="6"/>
-      <c r="E38" s="17" t="s">
-        <v>213</v>
+      <c r="E38" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G38" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G38" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H38" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Regla en PR #39; falta la pantalla</t>
+          <t xml:space="preserve">Regla en PR #39 y pantalla en PR #44</t>
         </is>
       </c>
     </row>
@@ -7453,14 +7630,24 @@
         <v>204</v>
       </c>
       <c r="D39" s="6"/>
-      <c r="E39" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="F39" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G39" s="19"/>
-      <c r="H39" s="17"/>
+      <c r="E39" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G39" s="19" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H39" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PR #44</t>
+        </is>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
@@ -7473,18 +7660,22 @@
         <v>204</v>
       </c>
       <c r="D40" s="6"/>
-      <c r="E40" s="17" t="s">
-        <v>213</v>
+      <c r="E40" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G40" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G40" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">El permiso de validador queda en el rol del perfil (PR #39); falta el selector</t>
+          <t xml:space="preserve">El permiso queda en el rol del perfil (PR #39); selector en PR #44</t>
         </is>
       </c>
     </row>
@@ -7499,14 +7690,24 @@
         <v>207</v>
       </c>
       <c r="D41" s="6"/>
-      <c r="E41" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G41" s="19"/>
-      <c r="H41" s="17"/>
+      <c r="E41" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G41" s="19" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H41" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PR #44</t>
+        </is>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
@@ -7519,14 +7720,24 @@
         <v>91</v>
       </c>
       <c r="D42" s="6"/>
-      <c r="E42" s="17" t="s">
-        <v>163</v>
-      </c>
-      <c r="F42" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G42" s="19"/>
-      <c r="H42" s="17"/>
+      <c r="E42" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matías Bustamante</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G42" s="19" t="n">
+        <v>46313</v>
+      </c>
+      <c r="H42" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RecyTrack_Casos_de_Prueba_S2.docx; redactados después del cierre del sprint</t>
+        </is>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
@@ -7539,14 +7750,22 @@
         <v>91</v>
       </c>
       <c r="D43" s="6"/>
-      <c r="E43" s="17" t="s">
-        <v>163</v>
-      </c>
-      <c r="F43" s="6" t="s">
-        <v>214</v>
+      <c r="E43" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matías Bustamante</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Por hacer</t>
+        </is>
       </c>
       <c r="G43" s="19"/>
-      <c r="H43" s="17"/>
+      <c r="H43" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En el S2 no se aprobaron pull requests (ver retrospectiva)</t>
+        </is>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
@@ -7559,18 +7778,22 @@
         <v>91</v>
       </c>
       <c r="D44" s="6"/>
-      <c r="E44" s="17" t="s">
-        <v>163</v>
+      <c r="E44" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matías Bustamante</t>
+        </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G44" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G44" s="19" t="n">
+        <v>46312</v>
+      </c>
       <c r="H44" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modelo de datos en PR #41</t>
+          <t xml:space="preserve">Modelo de datos en PR #41 y Modelo 4+1 en PR #52</t>
         </is>
       </c>
     </row>
@@ -7585,14 +7808,22 @@
         <v>91</v>
       </c>
       <c r="D45" s="6"/>
-      <c r="E45" s="17" t="s">
-        <v>163</v>
-      </c>
-      <c r="F45" s="6" t="s">
-        <v>214</v>
+      <c r="E45" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matías Bustamante</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En curso</t>
+        </is>
       </c>
       <c r="G45" s="19"/>
-      <c r="H45" s="17"/>
+      <c r="H45" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Demostración a la viña en curso</t>
+        </is>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
@@ -7605,14 +7836,24 @@
         <v>91</v>
       </c>
       <c r="D46" s="6"/>
-      <c r="E46" s="17" t="s">
-        <v>163</v>
-      </c>
-      <c r="F46" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G46" s="19"/>
-      <c r="H46" s="17"/>
+      <c r="E46" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matías Bustamante</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G46" s="19" t="n">
+        <v>46311</v>
+      </c>
+      <c r="H46" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retrospectiva del 16 de octubre (RecyTrack_Retrospectiva_S2.docx)</t>
+        </is>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
@@ -7865,13 +8106,19 @@
       <c r="D12" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E12" s="17"/>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G12" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H12" s="5" t="s">
         <v>268</v>
       </c>
@@ -7904,13 +8151,19 @@
       <c r="D13" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="17"/>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vicente Torres y Álvaro Jaña</t>
+        </is>
+      </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G13" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H13" s="5" t="s">
         <v>271</v>
       </c>
@@ -7943,13 +8196,19 @@
       <c r="D14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="17"/>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vicente Torres</t>
+        </is>
+      </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G14" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>46301</v>
+      </c>
       <c r="H14" s="5" t="s">
         <v>274</v>
       </c>
@@ -7982,13 +8241,19 @@
       <c r="D15" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E15" s="17"/>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G15" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G15" s="19" t="n">
+        <v>46301</v>
+      </c>
       <c r="H15" s="5" t="s">
         <v>277</v>
       </c>
@@ -8021,13 +8286,19 @@
       <c r="D16" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E16" s="17"/>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vicente Torres</t>
+        </is>
+      </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G16" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G16" s="19" t="n">
+        <v>46301</v>
+      </c>
       <c r="H16" s="5" t="s">
         <v>280</v>
       </c>
@@ -8060,13 +8331,19 @@
       <c r="D17" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E17" s="17"/>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G17" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G17" s="19" t="n">
+        <v>46301</v>
+      </c>
       <c r="H17" s="5" t="s">
         <v>283</v>
       </c>
@@ -8099,11 +8376,19 @@
       <c r="D18" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E18" s="17"/>
-      <c r="F18" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G18" s="19"/>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G18" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H18" s="5" t="s">
         <v>286</v>
       </c>
@@ -8136,11 +8421,19 @@
       <c r="D19" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E19" s="17"/>
-      <c r="F19" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G19" s="19"/>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G19" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H19" s="5" t="s">
         <v>289</v>
       </c>
@@ -8173,11 +8466,19 @@
       <c r="D20" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E20" s="17"/>
-      <c r="F20" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G20" s="19"/>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G20" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H20" s="5" t="s">
         <v>292</v>
       </c>
@@ -8643,13 +8944,19 @@
       <c r="D12" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="E12" s="17"/>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G12" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H12" s="5" t="s">
         <v>310</v>
       </c>
@@ -8682,13 +8989,19 @@
       <c r="D13" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="17"/>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vicente Torres y Álvaro Jaña</t>
+        </is>
+      </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G13" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>46301</v>
+      </c>
       <c r="H13" s="5" t="s">
         <v>313</v>
       </c>
@@ -8721,13 +9034,19 @@
       <c r="D14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="17"/>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vicente Torres</t>
+        </is>
+      </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G14" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>46301</v>
+      </c>
       <c r="H14" s="5" t="s">
         <v>316</v>
       </c>
@@ -8760,13 +9079,19 @@
       <c r="D15" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E15" s="17"/>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G15" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G15" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H15" s="5" t="s">
         <v>319</v>
       </c>
@@ -8873,13 +9198,19 @@
       <c r="D18" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E18" s="17"/>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G18" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G18" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H18" s="5" t="s">
         <v>328</v>
       </c>
@@ -8912,11 +9243,19 @@
       <c r="D19" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E19" s="17"/>
-      <c r="F19" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G19" s="19"/>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G19" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H19" s="5" t="s">
         <v>331</v>
       </c>
@@ -8949,13 +9288,19 @@
       <c r="D20" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E20" s="17"/>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G20" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G20" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H20" s="5" t="s">
         <v>334</v>
       </c>
@@ -9421,13 +9766,19 @@
       <c r="D12" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E12" s="17"/>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G12" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H12" s="5" t="s">
         <v>351</v>
       </c>
@@ -9460,13 +9811,19 @@
       <c r="D13" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E13" s="17"/>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G13" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H13" s="5" t="s">
         <v>354</v>
       </c>
@@ -9499,11 +9856,19 @@
       <c r="D14" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E14" s="17"/>
-      <c r="F14" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G14" s="19"/>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H14" s="5" t="s">
         <v>357</v>
       </c>
@@ -9536,11 +9901,19 @@
       <c r="D15" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E15" s="17"/>
-      <c r="F15" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G15" s="19"/>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G15" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H15" s="5" t="s">
         <v>360</v>
       </c>
@@ -9573,11 +9946,19 @@
       <c r="D16" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E16" s="17"/>
-      <c r="F16" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G16" s="19"/>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G16" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H16" s="5" t="s">
         <v>363</v>
       </c>
@@ -9610,11 +9991,19 @@
       <c r="D17" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="17"/>
-      <c r="F17" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G17" s="19"/>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G17" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H17" s="5" t="s">
         <v>367</v>
       </c>
@@ -9647,11 +10036,19 @@
       <c r="D18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="17"/>
-      <c r="F18" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G18" s="19"/>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G18" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H18" s="5" t="s">
         <v>370</v>
       </c>
@@ -10221,11 +10618,19 @@
       <c r="D14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="17"/>
-      <c r="F14" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G14" s="19"/>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H14" s="5" t="s">
         <v>393</v>
       </c>
@@ -10258,11 +10663,19 @@
       <c r="D15" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E15" s="17"/>
-      <c r="F15" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G15" s="19"/>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Álvaro Jaña</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G15" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H15" s="5" t="s">
         <v>396</v>
       </c>
@@ -10295,13 +10708,19 @@
       <c r="D16" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="17"/>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vicente Torres y Álvaro Jaña</t>
+        </is>
+      </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">En curso</t>
-        </is>
-      </c>
-      <c r="G16" s="19"/>
+          <t xml:space="preserve">Hecho</t>
+        </is>
+      </c>
+      <c r="G16" s="19" t="n">
+        <v>46302</v>
+      </c>
       <c r="H16" s="5" t="s">
         <v>399</v>
       </c>

</xml_diff>